<commit_message>
Correct Kanal classification in published Vis Bélica history
</commit_message>
<xml_diff>
--- a/public/downloads/power-ranking/2026-09/power_ranking_vis_belica_septiembre_2026_publico.xlsx
+++ b/public/downloads/power-ranking/2026-09/power_ranking_vis_belica_septiembre_2026_publico.xlsx
@@ -14,7 +14,7 @@
     <sheet name="Histórico Vis Bélica" sheetId="4" state="visible" r:id="rId6"/>
   </sheets>
   <definedNames>
-    <definedName function="false" hidden="true" localSheetId="3" name="_xlnm._FilterDatabase" vbProcedure="false">'Histórico Vis Bélica'!$A$3:$K$154</definedName>
+    <definedName function="false" hidden="true" localSheetId="3" name="_xlnm._FilterDatabase" vbProcedure="false">'Histórico Vis Bélica'!$A$3:$K$153</definedName>
     <definedName function="false" hidden="true" localSheetId="1" name="_xlnm._FilterDatabase" vbProcedure="false">'Power Ranking VB Septiembre'!$A$3:$G$120</definedName>
     <definedName function="false" hidden="true" localSheetId="0" name="_xlnm._FilterDatabase" vbProcedure="false">'Ranking Vis Bélica Septiembre'!$A$3:$H$48</definedName>
     <definedName function="false" hidden="true" localSheetId="2" name="_xlnm._FilterDatabase" vbProcedure="false">'Stats Vis Bélica Septiembre'!$A$3:$B$11</definedName>
@@ -29,7 +29,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="354" uniqueCount="188">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="353" uniqueCount="187">
   <si>
     <t xml:space="preserve">Ranking Vis Bélica Septiembre</t>
   </si>
@@ -536,9 +536,6 @@
   </si>
   <si>
     <t xml:space="preserve">Héroes Of Normandie</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Kanal</t>
   </si>
   <si>
     <t xml:space="preserve">Little Round Top</t>
@@ -5272,7 +5269,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:K154"/>
+  <dimension ref="A1:K153"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="8"/>
@@ -5406,10 +5403,10 @@
         <v>0</v>
       </c>
       <c r="D6" s="3" t="n">
-        <v>0.029</v>
+        <v>0.03</v>
       </c>
       <c r="E6" s="3" t="n">
-        <v>0.049</v>
+        <v>0.05</v>
       </c>
       <c r="F6" s="3" t="n">
         <v>0</v>
@@ -5428,7 +5425,7 @@
       </c>
       <c r="K6" s="3" t="n">
         <f aca="false">SUM(B6:I6)</f>
-        <v>0.11</v>
+        <v>0.112</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5517,7 +5514,7 @@
         <v>0</v>
       </c>
       <c r="E9" s="3" t="n">
-        <v>0.049</v>
+        <v>0.05</v>
       </c>
       <c r="F9" s="3" t="n">
         <v>0</v>
@@ -5536,7 +5533,7 @@
       </c>
       <c r="K9" s="3" t="n">
         <f aca="false">SUM(B9:I9)</f>
-        <v>0.049</v>
+        <v>0.05</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5586,7 +5583,7 @@
         <v>0</v>
       </c>
       <c r="D11" s="3" t="n">
-        <v>0.088</v>
+        <v>0.091</v>
       </c>
       <c r="E11" s="3" t="n">
         <v>0</v>
@@ -5608,7 +5605,7 @@
       </c>
       <c r="K11" s="3" t="n">
         <f aca="false">SUM(B11:I11)</f>
-        <v>0.088</v>
+        <v>0.091</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5838,7 +5835,7 @@
         <v>0</v>
       </c>
       <c r="D18" s="3" t="n">
-        <v>0.059</v>
+        <v>0.061</v>
       </c>
       <c r="E18" s="3" t="n">
         <v>0</v>
@@ -5860,7 +5857,7 @@
       </c>
       <c r="K18" s="3" t="n">
         <f aca="false">SUM(B18:I18)</f>
-        <v>0.059</v>
+        <v>0.061</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5949,7 +5946,7 @@
         <v>0</v>
       </c>
       <c r="E21" s="3" t="n">
-        <v>0.024</v>
+        <v>0.025</v>
       </c>
       <c r="F21" s="3" t="n">
         <v>0</v>
@@ -5968,7 +5965,7 @@
       </c>
       <c r="K21" s="3" t="n">
         <f aca="false">SUM(B21:I21)</f>
-        <v>0.024</v>
+        <v>0.025</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6021,7 +6018,7 @@
         <v>0</v>
       </c>
       <c r="E23" s="3" t="n">
-        <v>0.073</v>
+        <v>0.075</v>
       </c>
       <c r="F23" s="3" t="n">
         <v>0</v>
@@ -6040,7 +6037,7 @@
       </c>
       <c r="K23" s="3" t="n">
         <f aca="false">SUM(B23:I23)</f>
-        <v>0.073</v>
+        <v>0.075</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6057,7 +6054,7 @@
         <v>0</v>
       </c>
       <c r="E24" s="3" t="n">
-        <v>0.024</v>
+        <v>0.025</v>
       </c>
       <c r="F24" s="3" t="n">
         <v>0</v>
@@ -6076,7 +6073,7 @@
       </c>
       <c r="K24" s="3" t="n">
         <f aca="false">SUM(B24:I24)</f>
-        <v>0.024</v>
+        <v>0.025</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6126,10 +6123,10 @@
         <v>0</v>
       </c>
       <c r="D26" s="3" t="n">
-        <v>0.088</v>
+        <v>0.091</v>
       </c>
       <c r="E26" s="3" t="n">
-        <v>0.098</v>
+        <v>0.1</v>
       </c>
       <c r="F26" s="3" t="n">
         <v>0</v>
@@ -6148,7 +6145,7 @@
       </c>
       <c r="K26" s="3" t="n">
         <f aca="false">SUM(B26:I26)</f>
-        <v>0.186</v>
+        <v>0.191</v>
       </c>
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6156,16 +6153,16 @@
         <v>11</v>
       </c>
       <c r="B27" s="3" t="n">
-        <v>0.111</v>
+        <v>0.118</v>
       </c>
       <c r="C27" s="3" t="n">
-        <v>0.368</v>
+        <v>0.389</v>
       </c>
       <c r="D27" s="3" t="n">
-        <v>0.147</v>
+        <v>0.152</v>
       </c>
       <c r="E27" s="3" t="n">
-        <v>0.195</v>
+        <v>0.2</v>
       </c>
       <c r="F27" s="3" t="n">
         <v>0.077</v>
@@ -6184,7 +6181,7 @@
       </c>
       <c r="K27" s="3" t="n">
         <f aca="false">SUM(B27:I27)</f>
-        <v>1.254</v>
+        <v>1.292</v>
       </c>
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6201,7 +6198,7 @@
         <v>0</v>
       </c>
       <c r="E28" s="3" t="n">
-        <v>0.024</v>
+        <v>0.025</v>
       </c>
       <c r="F28" s="3" t="n">
         <v>0</v>
@@ -6220,7 +6217,7 @@
       </c>
       <c r="K28" s="3" t="n">
         <f aca="false">SUM(B28:I28)</f>
-        <v>0.024</v>
+        <v>0.025</v>
       </c>
     </row>
     <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6237,7 +6234,7 @@
         <v>0</v>
       </c>
       <c r="E29" s="3" t="n">
-        <v>0.049</v>
+        <v>0.05</v>
       </c>
       <c r="F29" s="3" t="n">
         <v>0</v>
@@ -6256,7 +6253,7 @@
       </c>
       <c r="K29" s="3" t="n">
         <f aca="false">SUM(B29:I29)</f>
-        <v>0.081</v>
+        <v>0.082</v>
       </c>
     </row>
     <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6345,7 +6342,7 @@
         <v>0</v>
       </c>
       <c r="E32" s="3" t="n">
-        <v>0.073</v>
+        <v>0.075</v>
       </c>
       <c r="F32" s="3" t="n">
         <v>0</v>
@@ -6364,7 +6361,7 @@
       </c>
       <c r="K32" s="3" t="n">
         <f aca="false">SUM(B32:I32)</f>
-        <v>0.121</v>
+        <v>0.123</v>
       </c>
     </row>
     <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6381,7 +6378,7 @@
         <v>0</v>
       </c>
       <c r="E33" s="3" t="n">
-        <v>0.073</v>
+        <v>0.075</v>
       </c>
       <c r="F33" s="3" t="n">
         <v>0</v>
@@ -6400,7 +6397,7 @@
       </c>
       <c r="K33" s="3" t="n">
         <f aca="false">SUM(B33:I33)</f>
-        <v>0.089</v>
+        <v>0.091</v>
       </c>
     </row>
     <row r="34" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6516,16 +6513,16 @@
         <v>15</v>
       </c>
       <c r="B37" s="3" t="n">
+        <v>0.059</v>
+      </c>
+      <c r="C37" s="3" t="n">
         <v>0.056</v>
       </c>
-      <c r="C37" s="3" t="n">
-        <v>0.053</v>
-      </c>
       <c r="D37" s="3" t="n">
         <v>0</v>
       </c>
       <c r="E37" s="3" t="n">
-        <v>0.073</v>
+        <v>0.075</v>
       </c>
       <c r="F37" s="3" t="n">
         <v>0.115</v>
@@ -6544,7 +6541,7 @@
       </c>
       <c r="K37" s="3" t="n">
         <f aca="false">SUM(B37:I37)</f>
-        <v>0.467</v>
+        <v>0.475</v>
       </c>
     </row>
     <row r="38" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6594,7 +6591,7 @@
         <v>0</v>
       </c>
       <c r="D39" s="3" t="n">
-        <v>0.059</v>
+        <v>0.061</v>
       </c>
       <c r="E39" s="3" t="n">
         <v>0</v>
@@ -6616,7 +6613,7 @@
       </c>
       <c r="K39" s="3" t="n">
         <f aca="false">SUM(B39:I39)</f>
-        <v>0.059</v>
+        <v>0.061</v>
       </c>
     </row>
     <row r="40" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6633,7 +6630,7 @@
         <v>0</v>
       </c>
       <c r="E40" s="3" t="n">
-        <v>0.024</v>
+        <v>0.025</v>
       </c>
       <c r="F40" s="3" t="n">
         <v>0</v>
@@ -6652,7 +6649,7 @@
       </c>
       <c r="K40" s="3" t="n">
         <f aca="false">SUM(B40:I40)</f>
-        <v>0.06</v>
+        <v>0.061</v>
       </c>
     </row>
     <row r="41" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6660,7 +6657,7 @@
         <v>63</v>
       </c>
       <c r="B41" s="3" t="n">
-        <v>0.167</v>
+        <v>0.176</v>
       </c>
       <c r="C41" s="3" t="n">
         <v>0</v>
@@ -6688,7 +6685,7 @@
       </c>
       <c r="K41" s="3" t="n">
         <f aca="false">SUM(B41:I41)</f>
-        <v>0.323</v>
+        <v>0.332</v>
       </c>
     </row>
     <row r="42" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6741,7 +6738,7 @@
         <v>0</v>
       </c>
       <c r="E43" s="3" t="n">
-        <v>0.049</v>
+        <v>0.05</v>
       </c>
       <c r="F43" s="3" t="n">
         <v>0</v>
@@ -6760,7 +6757,7 @@
       </c>
       <c r="K43" s="3" t="n">
         <f aca="false">SUM(B43:I43)</f>
-        <v>0.049</v>
+        <v>0.05</v>
       </c>
     </row>
     <row r="44" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6774,7 +6771,7 @@
         <v>0</v>
       </c>
       <c r="D44" s="3" t="n">
-        <v>0.059</v>
+        <v>0.061</v>
       </c>
       <c r="E44" s="3" t="n">
         <v>0</v>
@@ -6796,7 +6793,7 @@
       </c>
       <c r="K44" s="3" t="n">
         <f aca="false">SUM(B44:I44)</f>
-        <v>0.291</v>
+        <v>0.293</v>
       </c>
     </row>
     <row r="45" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6810,7 +6807,7 @@
         <v>0</v>
       </c>
       <c r="D45" s="3" t="n">
-        <v>0.029</v>
+        <v>0.03</v>
       </c>
       <c r="E45" s="3" t="n">
         <v>0</v>
@@ -6832,7 +6829,7 @@
       </c>
       <c r="K45" s="3" t="n">
         <f aca="false">SUM(B45:I45)</f>
-        <v>0.485</v>
+        <v>0.486</v>
       </c>
     </row>
     <row r="46" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6840,16 +6837,16 @@
         <v>9</v>
       </c>
       <c r="B46" s="3" t="n">
-        <v>1</v>
+        <v>1.059</v>
       </c>
       <c r="C46" s="3" t="n">
-        <v>0.632</v>
+        <v>0.667</v>
       </c>
       <c r="D46" s="3" t="n">
-        <v>0.294</v>
+        <v>0.303</v>
       </c>
       <c r="E46" s="3" t="n">
-        <v>0.537</v>
+        <v>0.55</v>
       </c>
       <c r="F46" s="3" t="n">
         <v>0.481</v>
@@ -6868,7 +6865,7 @@
       </c>
       <c r="K46" s="3" t="n">
         <f aca="false">SUM(B46:I46)</f>
-        <v>4.063</v>
+        <v>4.179</v>
       </c>
     </row>
     <row r="47" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6957,7 +6954,7 @@
         <v>0</v>
       </c>
       <c r="E49" s="3" t="n">
-        <v>0.073</v>
+        <v>0.075</v>
       </c>
       <c r="F49" s="3" t="n">
         <v>0</v>
@@ -6976,7 +6973,7 @@
       </c>
       <c r="K49" s="3" t="n">
         <f aca="false">SUM(B49:I49)</f>
-        <v>0.073</v>
+        <v>0.075</v>
       </c>
     </row>
     <row r="50" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6987,13 +6984,13 @@
         <v>0</v>
       </c>
       <c r="C50" s="3" t="n">
-        <v>0.211</v>
+        <v>0.222</v>
       </c>
       <c r="D50" s="3" t="n">
-        <v>0.118</v>
+        <v>0.121</v>
       </c>
       <c r="E50" s="3" t="n">
-        <v>0.024</v>
+        <v>0.025</v>
       </c>
       <c r="F50" s="3" t="n">
         <v>0.058</v>
@@ -7012,7 +7009,7 @@
       </c>
       <c r="K50" s="3" t="n">
         <f aca="false">SUM(B50:I50)</f>
-        <v>0.702</v>
+        <v>0.717</v>
       </c>
     </row>
     <row r="51" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -7026,10 +7023,10 @@
         <v>0</v>
       </c>
       <c r="D51" s="3" t="n">
-        <v>0.029</v>
+        <v>0.03</v>
       </c>
       <c r="E51" s="3" t="n">
-        <v>0.024</v>
+        <v>0.025</v>
       </c>
       <c r="F51" s="3" t="n">
         <v>0</v>
@@ -7048,7 +7045,7 @@
       </c>
       <c r="K51" s="3" t="n">
         <f aca="false">SUM(B51:I51)</f>
-        <v>0.053</v>
+        <v>0.055</v>
       </c>
     </row>
     <row r="52" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -7101,7 +7098,7 @@
         <v>0</v>
       </c>
       <c r="E53" s="3" t="n">
-        <v>0.073</v>
+        <v>0.075</v>
       </c>
       <c r="F53" s="3" t="n">
         <v>0</v>
@@ -7120,7 +7117,7 @@
       </c>
       <c r="K53" s="3" t="n">
         <f aca="false">SUM(B53:I53)</f>
-        <v>0.176</v>
+        <v>0.178</v>
       </c>
     </row>
     <row r="54" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -7137,7 +7134,7 @@
         <v>0</v>
       </c>
       <c r="E54" s="3" t="n">
-        <v>0.024</v>
+        <v>0.025</v>
       </c>
       <c r="F54" s="3" t="n">
         <v>0</v>
@@ -7156,7 +7153,7 @@
       </c>
       <c r="K54" s="3" t="n">
         <f aca="false">SUM(B54:I54)</f>
-        <v>0.142</v>
+        <v>0.143</v>
       </c>
     </row>
     <row r="55" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -7173,7 +7170,7 @@
         <v>0</v>
       </c>
       <c r="E55" s="3" t="n">
-        <v>0.073</v>
+        <v>0.075</v>
       </c>
       <c r="F55" s="3" t="n">
         <v>0</v>
@@ -7192,7 +7189,7 @@
       </c>
       <c r="K55" s="3" t="n">
         <f aca="false">SUM(B55:I55)</f>
-        <v>0.073</v>
+        <v>0.075</v>
       </c>
     </row>
     <row r="56" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -7209,7 +7206,7 @@
         <v>0</v>
       </c>
       <c r="E56" s="3" t="n">
-        <v>0.049</v>
+        <v>0.05</v>
       </c>
       <c r="F56" s="3" t="n">
         <v>0.154</v>
@@ -7228,7 +7225,7 @@
       </c>
       <c r="K56" s="3" t="n">
         <f aca="false">SUM(B56:I56)</f>
-        <v>0.725</v>
+        <v>0.726</v>
       </c>
     </row>
     <row r="57" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -7278,7 +7275,7 @@
         <v>0</v>
       </c>
       <c r="D58" s="3" t="n">
-        <v>0.029</v>
+        <v>0.03</v>
       </c>
       <c r="E58" s="3" t="n">
         <v>0</v>
@@ -7300,7 +7297,7 @@
       </c>
       <c r="K58" s="3" t="n">
         <f aca="false">SUM(B58:I58)</f>
-        <v>0.294</v>
+        <v>0.295</v>
       </c>
     </row>
     <row r="59" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -7347,13 +7344,13 @@
         <v>0</v>
       </c>
       <c r="C60" s="3" t="n">
-        <v>0.105</v>
+        <v>0.111</v>
       </c>
       <c r="D60" s="3" t="n">
-        <v>0.265</v>
+        <v>0.273</v>
       </c>
       <c r="E60" s="3" t="n">
-        <v>0.22</v>
+        <v>0.225</v>
       </c>
       <c r="F60" s="3" t="n">
         <v>0.077</v>
@@ -7372,7 +7369,7 @@
       </c>
       <c r="K60" s="3" t="n">
         <f aca="false">SUM(B60:I60)</f>
-        <v>1.232</v>
+        <v>1.251</v>
       </c>
     </row>
     <row r="61" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -7458,7 +7455,7 @@
         <v>0</v>
       </c>
       <c r="D63" s="3" t="n">
-        <v>0.029</v>
+        <v>0.03</v>
       </c>
       <c r="E63" s="3" t="n">
         <v>0</v>
@@ -7480,7 +7477,7 @@
       </c>
       <c r="K63" s="3" t="n">
         <f aca="false">SUM(B63:I63)</f>
-        <v>0.029</v>
+        <v>0.03</v>
       </c>
     </row>
     <row r="64" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -7497,7 +7494,7 @@
         <v>0</v>
       </c>
       <c r="E64" s="3" t="n">
-        <v>0.073</v>
+        <v>0.075</v>
       </c>
       <c r="F64" s="3" t="n">
         <v>0.019</v>
@@ -7516,7 +7513,7 @@
       </c>
       <c r="K64" s="3" t="n">
         <f aca="false">SUM(B64:I64)</f>
-        <v>0.092</v>
+        <v>0.094</v>
       </c>
     </row>
     <row r="65" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -7602,10 +7599,10 @@
         <v>0</v>
       </c>
       <c r="D67" s="3" t="n">
-        <v>0.088</v>
+        <v>0.091</v>
       </c>
       <c r="E67" s="3" t="n">
-        <v>0.073</v>
+        <v>0.075</v>
       </c>
       <c r="F67" s="3" t="n">
         <v>0</v>
@@ -7624,7 +7621,7 @@
       </c>
       <c r="K67" s="3" t="n">
         <f aca="false">SUM(B67:I67)</f>
-        <v>0.216</v>
+        <v>0.221</v>
       </c>
     </row>
     <row r="68" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -7671,10 +7668,10 @@
         <v>0</v>
       </c>
       <c r="C69" s="3" t="n">
-        <v>0.158</v>
+        <v>0.167</v>
       </c>
       <c r="D69" s="3" t="n">
-        <v>0.059</v>
+        <v>0.061</v>
       </c>
       <c r="E69" s="3" t="n">
         <v>0</v>
@@ -7696,7 +7693,7 @@
       </c>
       <c r="K69" s="3" t="n">
         <f aca="false">SUM(B69:I69)</f>
-        <v>0.374</v>
+        <v>0.385</v>
       </c>
     </row>
     <row r="70" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -7710,7 +7707,7 @@
         <v>0</v>
       </c>
       <c r="D70" s="3" t="n">
-        <v>0.059</v>
+        <v>0.061</v>
       </c>
       <c r="E70" s="3" t="n">
         <v>0</v>
@@ -7732,7 +7729,7 @@
       </c>
       <c r="K70" s="3" t="n">
         <f aca="false">SUM(B70:I70)</f>
-        <v>0.075</v>
+        <v>0.077</v>
       </c>
     </row>
     <row r="71" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -7749,7 +7746,7 @@
         <v>0</v>
       </c>
       <c r="E71" s="3" t="n">
-        <v>0.024</v>
+        <v>0.025</v>
       </c>
       <c r="F71" s="3" t="n">
         <v>0</v>
@@ -7768,7 +7765,7 @@
       </c>
       <c r="K71" s="3" t="n">
         <f aca="false">SUM(B71:I71)</f>
-        <v>0.024</v>
+        <v>0.025</v>
       </c>
     </row>
     <row r="72" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -7782,7 +7779,7 @@
         <v>0</v>
       </c>
       <c r="D72" s="3" t="n">
-        <v>0.147</v>
+        <v>0.152</v>
       </c>
       <c r="E72" s="3" t="n">
         <v>0</v>
@@ -7804,7 +7801,7 @@
       </c>
       <c r="K72" s="3" t="n">
         <f aca="false">SUM(B72:I72)</f>
-        <v>0.312</v>
+        <v>0.317</v>
       </c>
     </row>
     <row r="73" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -7848,7 +7845,7 @@
         <v>107</v>
       </c>
       <c r="B74" s="3" t="n">
-        <v>0.111</v>
+        <v>0.118</v>
       </c>
       <c r="C74" s="3" t="n">
         <v>0</v>
@@ -7857,7 +7854,7 @@
         <v>0</v>
       </c>
       <c r="E74" s="3" t="n">
-        <v>0.024</v>
+        <v>0.025</v>
       </c>
       <c r="F74" s="3" t="n">
         <v>0.058</v>
@@ -7876,24 +7873,24 @@
       </c>
       <c r="K74" s="3" t="n">
         <f aca="false">SUM(B74:I74)</f>
-        <v>0.193</v>
+        <v>0.201</v>
       </c>
     </row>
     <row r="75" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A75" s="0" t="s">
-        <v>169</v>
+        <v>89</v>
       </c>
       <c r="B75" s="3" t="n">
-        <v>0.167</v>
+        <v>0</v>
       </c>
       <c r="C75" s="3" t="n">
-        <v>0.053</v>
+        <v>0</v>
       </c>
       <c r="D75" s="3" t="n">
-        <v>0.059</v>
+        <v>0</v>
       </c>
       <c r="E75" s="3" t="n">
-        <v>0.024</v>
+        <v>0</v>
       </c>
       <c r="F75" s="3" t="n">
         <v>0</v>
@@ -7902,22 +7899,22 @@
         <v>0</v>
       </c>
       <c r="H75" s="3" t="n">
-        <v>0</v>
+        <v>0.032</v>
       </c>
       <c r="I75" s="3" t="n">
         <v>0</v>
       </c>
       <c r="J75" s="4" t="n">
-        <v>0</v>
+        <v>0.0048</v>
       </c>
       <c r="K75" s="3" t="n">
         <f aca="false">SUM(B75:I75)</f>
-        <v>0.303</v>
+        <v>0.032</v>
       </c>
     </row>
     <row r="76" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A76" s="0" t="s">
-        <v>89</v>
+        <v>116</v>
       </c>
       <c r="B76" s="3" t="n">
         <v>0</v>
@@ -7938,22 +7935,22 @@
         <v>0</v>
       </c>
       <c r="H76" s="3" t="n">
-        <v>0.032</v>
+        <v>0.016</v>
       </c>
       <c r="I76" s="3" t="n">
         <v>0</v>
       </c>
       <c r="J76" s="4" t="n">
-        <v>0.0048</v>
+        <v>0.0024</v>
       </c>
       <c r="K76" s="3" t="n">
         <f aca="false">SUM(B76:I76)</f>
-        <v>0.032</v>
+        <v>0.016</v>
       </c>
     </row>
     <row r="77" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A77" s="0" t="s">
-        <v>116</v>
+        <v>69</v>
       </c>
       <c r="B77" s="3" t="n">
         <v>0</v>
@@ -7971,25 +7968,25 @@
         <v>0</v>
       </c>
       <c r="G77" s="3" t="n">
-        <v>0</v>
+        <v>0.023</v>
       </c>
       <c r="H77" s="3" t="n">
-        <v>0.016</v>
+        <v>0.048</v>
       </c>
       <c r="I77" s="3" t="n">
         <v>0</v>
       </c>
       <c r="J77" s="4" t="n">
-        <v>0.0024</v>
+        <v>0.00927</v>
       </c>
       <c r="K77" s="3" t="n">
         <f aca="false">SUM(B77:I77)</f>
-        <v>0.016</v>
+        <v>0.071</v>
       </c>
     </row>
     <row r="78" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A78" s="0" t="s">
-        <v>69</v>
+        <v>169</v>
       </c>
       <c r="B78" s="3" t="n">
         <v>0</v>
@@ -8001,31 +7998,31 @@
         <v>0</v>
       </c>
       <c r="E78" s="3" t="n">
-        <v>0</v>
+        <v>0.05</v>
       </c>
       <c r="F78" s="3" t="n">
         <v>0</v>
       </c>
       <c r="G78" s="3" t="n">
-        <v>0.023</v>
+        <v>0</v>
       </c>
       <c r="H78" s="3" t="n">
-        <v>0.048</v>
+        <v>0</v>
       </c>
       <c r="I78" s="3" t="n">
         <v>0</v>
       </c>
       <c r="J78" s="4" t="n">
-        <v>0.00927</v>
+        <v>0</v>
       </c>
       <c r="K78" s="3" t="n">
         <f aca="false">SUM(B78:I78)</f>
-        <v>0.071</v>
+        <v>0.05</v>
       </c>
     </row>
     <row r="79" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A79" s="0" t="s">
-        <v>170</v>
+        <v>38</v>
       </c>
       <c r="B79" s="3" t="n">
         <v>0</v>
@@ -8037,7 +8034,7 @@
         <v>0</v>
       </c>
       <c r="E79" s="3" t="n">
-        <v>0.049</v>
+        <v>0.025</v>
       </c>
       <c r="F79" s="3" t="n">
         <v>0</v>
@@ -8046,22 +8043,22 @@
         <v>0</v>
       </c>
       <c r="H79" s="3" t="n">
-        <v>0</v>
+        <v>0.032</v>
       </c>
       <c r="I79" s="3" t="n">
-        <v>0</v>
+        <v>0.036</v>
       </c>
       <c r="J79" s="4" t="n">
-        <v>0</v>
+        <v>0.03</v>
       </c>
       <c r="K79" s="3" t="n">
         <f aca="false">SUM(B79:I79)</f>
-        <v>0.049</v>
+        <v>0.093</v>
       </c>
     </row>
     <row r="80" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A80" s="0" t="s">
-        <v>38</v>
+        <v>48</v>
       </c>
       <c r="B80" s="3" t="n">
         <v>0</v>
@@ -8073,7 +8070,7 @@
         <v>0</v>
       </c>
       <c r="E80" s="3" t="n">
-        <v>0.024</v>
+        <v>0</v>
       </c>
       <c r="F80" s="3" t="n">
         <v>0</v>
@@ -8082,94 +8079,94 @@
         <v>0</v>
       </c>
       <c r="H80" s="3" t="n">
-        <v>0.032</v>
+        <v>0</v>
       </c>
       <c r="I80" s="3" t="n">
-        <v>0.036</v>
+        <v>0.018</v>
       </c>
       <c r="J80" s="4" t="n">
-        <v>0.03</v>
+        <v>0.0126</v>
       </c>
       <c r="K80" s="3" t="n">
         <f aca="false">SUM(B80:I80)</f>
-        <v>0.092</v>
+        <v>0.018</v>
       </c>
     </row>
     <row r="81" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A81" s="0" t="s">
-        <v>48</v>
+        <v>68</v>
       </c>
       <c r="B81" s="3" t="n">
-        <v>0</v>
+        <v>0.706</v>
       </c>
       <c r="C81" s="3" t="n">
-        <v>0</v>
+        <v>0.111</v>
       </c>
       <c r="D81" s="3" t="n">
-        <v>0</v>
+        <v>0.152</v>
       </c>
       <c r="E81" s="3" t="n">
-        <v>0</v>
+        <v>0.075</v>
       </c>
       <c r="F81" s="3" t="n">
         <v>0</v>
       </c>
       <c r="G81" s="3" t="n">
-        <v>0</v>
+        <v>0.093</v>
       </c>
       <c r="H81" s="3" t="n">
-        <v>0</v>
+        <v>0.016</v>
       </c>
       <c r="I81" s="3" t="n">
-        <v>0.018</v>
+        <v>0</v>
       </c>
       <c r="J81" s="4" t="n">
-        <v>0.0126</v>
+        <v>0.01077</v>
       </c>
       <c r="K81" s="3" t="n">
         <f aca="false">SUM(B81:I81)</f>
-        <v>0.018</v>
+        <v>1.153</v>
       </c>
     </row>
     <row r="82" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A82" s="0" t="s">
-        <v>68</v>
+        <v>170</v>
       </c>
       <c r="B82" s="3" t="n">
-        <v>0.667</v>
+        <v>0</v>
       </c>
       <c r="C82" s="3" t="n">
-        <v>0.105</v>
+        <v>0</v>
       </c>
       <c r="D82" s="3" t="n">
-        <v>0.147</v>
+        <v>0</v>
       </c>
       <c r="E82" s="3" t="n">
-        <v>0.073</v>
+        <v>0.075</v>
       </c>
       <c r="F82" s="3" t="n">
         <v>0</v>
       </c>
       <c r="G82" s="3" t="n">
-        <v>0.093</v>
+        <v>0</v>
       </c>
       <c r="H82" s="3" t="n">
-        <v>0.016</v>
+        <v>0</v>
       </c>
       <c r="I82" s="3" t="n">
         <v>0</v>
       </c>
       <c r="J82" s="4" t="n">
-        <v>0.01077</v>
+        <v>0</v>
       </c>
       <c r="K82" s="3" t="n">
         <f aca="false">SUM(B82:I82)</f>
-        <v>1.101</v>
+        <v>0.075</v>
       </c>
     </row>
     <row r="83" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A83" s="0" t="s">
-        <v>171</v>
+        <v>90</v>
       </c>
       <c r="B83" s="3" t="n">
         <v>0</v>
@@ -8181,7 +8178,7 @@
         <v>0</v>
       </c>
       <c r="E83" s="3" t="n">
-        <v>0.073</v>
+        <v>0</v>
       </c>
       <c r="F83" s="3" t="n">
         <v>0</v>
@@ -8190,22 +8187,22 @@
         <v>0</v>
       </c>
       <c r="H83" s="3" t="n">
-        <v>0</v>
+        <v>0.032</v>
       </c>
       <c r="I83" s="3" t="n">
         <v>0</v>
       </c>
       <c r="J83" s="4" t="n">
-        <v>0</v>
+        <v>0.0048</v>
       </c>
       <c r="K83" s="3" t="n">
         <f aca="false">SUM(B83:I83)</f>
-        <v>0.073</v>
+        <v>0.032</v>
       </c>
     </row>
     <row r="84" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A84" s="0" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="B84" s="3" t="n">
         <v>0</v>
@@ -8241,7 +8238,7 @@
     </row>
     <row r="85" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A85" s="0" t="s">
-        <v>91</v>
+        <v>171</v>
       </c>
       <c r="B85" s="3" t="n">
         <v>0</v>
@@ -8250,7 +8247,7 @@
         <v>0</v>
       </c>
       <c r="D85" s="3" t="n">
-        <v>0</v>
+        <v>0.091</v>
       </c>
       <c r="E85" s="3" t="n">
         <v>0</v>
@@ -8262,22 +8259,22 @@
         <v>0</v>
       </c>
       <c r="H85" s="3" t="n">
-        <v>0.032</v>
+        <v>0</v>
       </c>
       <c r="I85" s="3" t="n">
         <v>0</v>
       </c>
       <c r="J85" s="4" t="n">
-        <v>0.0048</v>
+        <v>0</v>
       </c>
       <c r="K85" s="3" t="n">
         <f aca="false">SUM(B85:I85)</f>
-        <v>0.032</v>
+        <v>0.091</v>
       </c>
     </row>
     <row r="86" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A86" s="0" t="s">
-        <v>172</v>
+        <v>22</v>
       </c>
       <c r="B86" s="3" t="n">
         <v>0</v>
@@ -8286,7 +8283,7 @@
         <v>0</v>
       </c>
       <c r="D86" s="3" t="n">
-        <v>0.088</v>
+        <v>0</v>
       </c>
       <c r="E86" s="3" t="n">
         <v>0</v>
@@ -8301,19 +8298,19 @@
         <v>0</v>
       </c>
       <c r="I86" s="3" t="n">
-        <v>0</v>
+        <v>0.055</v>
       </c>
       <c r="J86" s="4" t="n">
-        <v>0</v>
+        <v>0.0385</v>
       </c>
       <c r="K86" s="3" t="n">
         <f aca="false">SUM(B86:I86)</f>
-        <v>0.088</v>
+        <v>0.055</v>
       </c>
     </row>
     <row r="87" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A87" s="0" t="s">
-        <v>22</v>
+        <v>121</v>
       </c>
       <c r="B87" s="3" t="n">
         <v>0</v>
@@ -8328,7 +8325,7 @@
         <v>0</v>
       </c>
       <c r="F87" s="3" t="n">
-        <v>0</v>
+        <v>0.038</v>
       </c>
       <c r="G87" s="3" t="n">
         <v>0</v>
@@ -8337,19 +8334,19 @@
         <v>0</v>
       </c>
       <c r="I87" s="3" t="n">
-        <v>0.055</v>
+        <v>0</v>
       </c>
       <c r="J87" s="4" t="n">
-        <v>0.0385</v>
+        <v>0.00228</v>
       </c>
       <c r="K87" s="3" t="n">
         <f aca="false">SUM(B87:I87)</f>
-        <v>0.055</v>
+        <v>0.038</v>
       </c>
     </row>
     <row r="88" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A88" s="0" t="s">
-        <v>121</v>
+        <v>39</v>
       </c>
       <c r="B88" s="3" t="n">
         <v>0</v>
@@ -8364,28 +8361,28 @@
         <v>0</v>
       </c>
       <c r="F88" s="3" t="n">
-        <v>0.038</v>
+        <v>0</v>
       </c>
       <c r="G88" s="3" t="n">
-        <v>0</v>
+        <v>0.023</v>
       </c>
       <c r="H88" s="3" t="n">
-        <v>0</v>
+        <v>0.032</v>
       </c>
       <c r="I88" s="3" t="n">
-        <v>0</v>
+        <v>0.036</v>
       </c>
       <c r="J88" s="4" t="n">
-        <v>0.00228</v>
+        <v>0.03207</v>
       </c>
       <c r="K88" s="3" t="n">
         <f aca="false">SUM(B88:I88)</f>
-        <v>0.038</v>
+        <v>0.091</v>
       </c>
     </row>
     <row r="89" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A89" s="0" t="s">
-        <v>39</v>
+        <v>126</v>
       </c>
       <c r="B89" s="3" t="n">
         <v>0</v>
@@ -8406,22 +8403,22 @@
         <v>0.023</v>
       </c>
       <c r="H89" s="3" t="n">
-        <v>0.032</v>
+        <v>0</v>
       </c>
       <c r="I89" s="3" t="n">
-        <v>0.036</v>
+        <v>0</v>
       </c>
       <c r="J89" s="4" t="n">
-        <v>0.03207</v>
+        <v>0.00207</v>
       </c>
       <c r="K89" s="3" t="n">
         <f aca="false">SUM(B89:I89)</f>
-        <v>0.091</v>
+        <v>0.023</v>
       </c>
     </row>
     <row r="90" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A90" s="0" t="s">
-        <v>126</v>
+        <v>127</v>
       </c>
       <c r="B90" s="3" t="n">
         <v>0</v>
@@ -8457,7 +8454,7 @@
     </row>
     <row r="91" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A91" s="0" t="s">
-        <v>127</v>
+        <v>23</v>
       </c>
       <c r="B91" s="3" t="n">
         <v>0</v>
@@ -8472,28 +8469,28 @@
         <v>0</v>
       </c>
       <c r="F91" s="3" t="n">
-        <v>0</v>
+        <v>0.019</v>
       </c>
       <c r="G91" s="3" t="n">
-        <v>0.023</v>
+        <v>0</v>
       </c>
       <c r="H91" s="3" t="n">
-        <v>0</v>
+        <v>0.048</v>
       </c>
       <c r="I91" s="3" t="n">
-        <v>0</v>
+        <v>0.055</v>
       </c>
       <c r="J91" s="4" t="n">
-        <v>0.00207</v>
+        <v>0.04684</v>
       </c>
       <c r="K91" s="3" t="n">
         <f aca="false">SUM(B91:I91)</f>
-        <v>0.023</v>
+        <v>0.122</v>
       </c>
     </row>
     <row r="92" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A92" s="0" t="s">
-        <v>23</v>
+        <v>122</v>
       </c>
       <c r="B92" s="3" t="n">
         <v>0</v>
@@ -8508,28 +8505,28 @@
         <v>0</v>
       </c>
       <c r="F92" s="3" t="n">
-        <v>0.019</v>
+        <v>0.038</v>
       </c>
       <c r="G92" s="3" t="n">
         <v>0</v>
       </c>
       <c r="H92" s="3" t="n">
-        <v>0.048</v>
+        <v>0</v>
       </c>
       <c r="I92" s="3" t="n">
-        <v>0.055</v>
+        <v>0</v>
       </c>
       <c r="J92" s="4" t="n">
-        <v>0.04684</v>
+        <v>0.00228</v>
       </c>
       <c r="K92" s="3" t="n">
         <f aca="false">SUM(B92:I92)</f>
-        <v>0.122</v>
+        <v>0.038</v>
       </c>
     </row>
     <row r="93" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A93" s="0" t="s">
-        <v>122</v>
+        <v>24</v>
       </c>
       <c r="B93" s="3" t="n">
         <v>0</v>
@@ -8547,25 +8544,25 @@
         <v>0.038</v>
       </c>
       <c r="G93" s="3" t="n">
-        <v>0</v>
+        <v>0.047</v>
       </c>
       <c r="H93" s="3" t="n">
-        <v>0</v>
+        <v>0.048</v>
       </c>
       <c r="I93" s="3" t="n">
-        <v>0</v>
+        <v>0.055</v>
       </c>
       <c r="J93" s="4" t="n">
-        <v>0.00228</v>
+        <v>0.05221</v>
       </c>
       <c r="K93" s="3" t="n">
         <f aca="false">SUM(B93:I93)</f>
-        <v>0.038</v>
+        <v>0.188</v>
       </c>
     </row>
     <row r="94" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A94" s="0" t="s">
-        <v>24</v>
+        <v>172</v>
       </c>
       <c r="B94" s="3" t="n">
         <v>0</v>
@@ -8577,31 +8574,31 @@
         <v>0</v>
       </c>
       <c r="E94" s="3" t="n">
-        <v>0</v>
+        <v>0.025</v>
       </c>
       <c r="F94" s="3" t="n">
-        <v>0.038</v>
+        <v>0</v>
       </c>
       <c r="G94" s="3" t="n">
-        <v>0.047</v>
+        <v>0</v>
       </c>
       <c r="H94" s="3" t="n">
-        <v>0.048</v>
+        <v>0</v>
       </c>
       <c r="I94" s="3" t="n">
-        <v>0.055</v>
+        <v>0</v>
       </c>
       <c r="J94" s="4" t="n">
-        <v>0.05221</v>
+        <v>0</v>
       </c>
       <c r="K94" s="3" t="n">
         <f aca="false">SUM(B94:I94)</f>
-        <v>0.188</v>
+        <v>0.025</v>
       </c>
     </row>
     <row r="95" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A95" s="0" t="s">
-        <v>173</v>
+        <v>49</v>
       </c>
       <c r="B95" s="3" t="n">
         <v>0</v>
@@ -8613,31 +8610,31 @@
         <v>0</v>
       </c>
       <c r="E95" s="3" t="n">
-        <v>0.024</v>
+        <v>0.025</v>
       </c>
       <c r="F95" s="3" t="n">
-        <v>0</v>
+        <v>0.173</v>
       </c>
       <c r="G95" s="3" t="n">
-        <v>0</v>
+        <v>0.023</v>
       </c>
       <c r="H95" s="3" t="n">
-        <v>0</v>
+        <v>0.032</v>
       </c>
       <c r="I95" s="3" t="n">
-        <v>0</v>
+        <v>0.018</v>
       </c>
       <c r="J95" s="4" t="n">
-        <v>0</v>
+        <v>0.02985</v>
       </c>
       <c r="K95" s="3" t="n">
         <f aca="false">SUM(B95:I95)</f>
-        <v>0.024</v>
+        <v>0.271</v>
       </c>
     </row>
     <row r="96" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A96" s="0" t="s">
-        <v>49</v>
+        <v>131</v>
       </c>
       <c r="B96" s="3" t="n">
         <v>0</v>
@@ -8649,31 +8646,31 @@
         <v>0</v>
       </c>
       <c r="E96" s="3" t="n">
-        <v>0.024</v>
+        <v>0</v>
       </c>
       <c r="F96" s="3" t="n">
-        <v>0.173</v>
+        <v>0.019</v>
       </c>
       <c r="G96" s="3" t="n">
-        <v>0.023</v>
+        <v>0</v>
       </c>
       <c r="H96" s="3" t="n">
-        <v>0.032</v>
+        <v>0</v>
       </c>
       <c r="I96" s="3" t="n">
-        <v>0.018</v>
+        <v>0</v>
       </c>
       <c r="J96" s="4" t="n">
-        <v>0.02985</v>
+        <v>0.00114</v>
       </c>
       <c r="K96" s="3" t="n">
         <f aca="false">SUM(B96:I96)</f>
-        <v>0.27</v>
+        <v>0.019</v>
       </c>
     </row>
     <row r="97" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A97" s="0" t="s">
-        <v>131</v>
+        <v>71</v>
       </c>
       <c r="B97" s="3" t="n">
         <v>0</v>
@@ -8682,7 +8679,7 @@
         <v>0</v>
       </c>
       <c r="D97" s="3" t="n">
-        <v>0</v>
+        <v>0.03</v>
       </c>
       <c r="E97" s="3" t="n">
         <v>0</v>
@@ -8691,7 +8688,7 @@
         <v>0.019</v>
       </c>
       <c r="G97" s="3" t="n">
-        <v>0</v>
+        <v>0.07</v>
       </c>
       <c r="H97" s="3" t="n">
         <v>0</v>
@@ -8700,16 +8697,16 @@
         <v>0</v>
       </c>
       <c r="J97" s="4" t="n">
-        <v>0.00114</v>
+        <v>0.00744</v>
       </c>
       <c r="K97" s="3" t="n">
         <f aca="false">SUM(B97:I97)</f>
-        <v>0.019</v>
+        <v>0.119</v>
       </c>
     </row>
     <row r="98" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A98" s="0" t="s">
-        <v>71</v>
+        <v>76</v>
       </c>
       <c r="B98" s="3" t="n">
         <v>0</v>
@@ -8718,34 +8715,34 @@
         <v>0</v>
       </c>
       <c r="D98" s="3" t="n">
-        <v>0.029</v>
+        <v>0.061</v>
       </c>
       <c r="E98" s="3" t="n">
         <v>0</v>
       </c>
       <c r="F98" s="3" t="n">
-        <v>0.019</v>
+        <v>0</v>
       </c>
       <c r="G98" s="3" t="n">
-        <v>0.07</v>
+        <v>0</v>
       </c>
       <c r="H98" s="3" t="n">
-        <v>0</v>
+        <v>0.048</v>
       </c>
       <c r="I98" s="3" t="n">
         <v>0</v>
       </c>
       <c r="J98" s="4" t="n">
-        <v>0.00744</v>
+        <v>0.0072</v>
       </c>
       <c r="K98" s="3" t="n">
         <f aca="false">SUM(B98:I98)</f>
-        <v>0.118</v>
+        <v>0.109</v>
       </c>
     </row>
     <row r="99" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A99" s="0" t="s">
-        <v>76</v>
+        <v>173</v>
       </c>
       <c r="B99" s="3" t="n">
         <v>0</v>
@@ -8754,10 +8751,10 @@
         <v>0</v>
       </c>
       <c r="D99" s="3" t="n">
-        <v>0.059</v>
+        <v>0</v>
       </c>
       <c r="E99" s="3" t="n">
-        <v>0</v>
+        <v>0.025</v>
       </c>
       <c r="F99" s="3" t="n">
         <v>0</v>
@@ -8766,22 +8763,22 @@
         <v>0</v>
       </c>
       <c r="H99" s="3" t="n">
-        <v>0.048</v>
+        <v>0</v>
       </c>
       <c r="I99" s="3" t="n">
         <v>0</v>
       </c>
       <c r="J99" s="4" t="n">
-        <v>0.0072</v>
+        <v>0</v>
       </c>
       <c r="K99" s="3" t="n">
         <f aca="false">SUM(B99:I99)</f>
-        <v>0.107</v>
+        <v>0.025</v>
       </c>
     </row>
     <row r="100" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A100" s="0" t="s">
-        <v>174</v>
+        <v>40</v>
       </c>
       <c r="B100" s="3" t="n">
         <v>0</v>
@@ -8793,31 +8790,31 @@
         <v>0</v>
       </c>
       <c r="E100" s="3" t="n">
-        <v>0.024</v>
+        <v>0.075</v>
       </c>
       <c r="F100" s="3" t="n">
-        <v>0</v>
+        <v>0.058</v>
       </c>
       <c r="G100" s="3" t="n">
-        <v>0</v>
+        <v>0.047</v>
       </c>
       <c r="H100" s="3" t="n">
-        <v>0</v>
+        <v>0.032</v>
       </c>
       <c r="I100" s="3" t="n">
-        <v>0</v>
+        <v>0.036</v>
       </c>
       <c r="J100" s="4" t="n">
-        <v>0</v>
+        <v>0.03771</v>
       </c>
       <c r="K100" s="3" t="n">
         <f aca="false">SUM(B100:I100)</f>
-        <v>0.024</v>
+        <v>0.248</v>
       </c>
     </row>
     <row r="101" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A101" s="0" t="s">
-        <v>40</v>
+        <v>103</v>
       </c>
       <c r="B101" s="3" t="n">
         <v>0</v>
@@ -8829,37 +8826,37 @@
         <v>0</v>
       </c>
       <c r="E101" s="3" t="n">
-        <v>0.073</v>
+        <v>0</v>
       </c>
       <c r="F101" s="3" t="n">
-        <v>0.058</v>
+        <v>0</v>
       </c>
       <c r="G101" s="3" t="n">
         <v>0.047</v>
       </c>
       <c r="H101" s="3" t="n">
-        <v>0.032</v>
+        <v>0</v>
       </c>
       <c r="I101" s="3" t="n">
-        <v>0.036</v>
+        <v>0</v>
       </c>
       <c r="J101" s="4" t="n">
-        <v>0.03771</v>
+        <v>0.00423</v>
       </c>
       <c r="K101" s="3" t="n">
         <f aca="false">SUM(B101:I101)</f>
-        <v>0.246</v>
+        <v>0.047</v>
       </c>
     </row>
     <row r="102" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A102" s="0" t="s">
-        <v>103</v>
+        <v>65</v>
       </c>
       <c r="B102" s="3" t="n">
-        <v>0</v>
+        <v>0.176</v>
       </c>
       <c r="C102" s="3" t="n">
-        <v>0</v>
+        <v>0.167</v>
       </c>
       <c r="D102" s="3" t="n">
         <v>0</v>
@@ -8868,34 +8865,34 @@
         <v>0</v>
       </c>
       <c r="F102" s="3" t="n">
-        <v>0</v>
+        <v>0.038</v>
       </c>
       <c r="G102" s="3" t="n">
-        <v>0.047</v>
+        <v>0.093</v>
       </c>
       <c r="H102" s="3" t="n">
-        <v>0</v>
+        <v>0.032</v>
       </c>
       <c r="I102" s="3" t="n">
         <v>0</v>
       </c>
       <c r="J102" s="4" t="n">
-        <v>0.00423</v>
+        <v>0.01545</v>
       </c>
       <c r="K102" s="3" t="n">
         <f aca="false">SUM(B102:I102)</f>
-        <v>0.047</v>
+        <v>0.506</v>
       </c>
     </row>
     <row r="103" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A103" s="0" t="s">
-        <v>65</v>
+        <v>92</v>
       </c>
       <c r="B103" s="3" t="n">
-        <v>0.167</v>
+        <v>0</v>
       </c>
       <c r="C103" s="3" t="n">
-        <v>0.158</v>
+        <v>0</v>
       </c>
       <c r="D103" s="3" t="n">
         <v>0</v>
@@ -8904,10 +8901,10 @@
         <v>0</v>
       </c>
       <c r="F103" s="3" t="n">
-        <v>0.038</v>
+        <v>0</v>
       </c>
       <c r="G103" s="3" t="n">
-        <v>0.093</v>
+        <v>0</v>
       </c>
       <c r="H103" s="3" t="n">
         <v>0.032</v>
@@ -8916,16 +8913,16 @@
         <v>0</v>
       </c>
       <c r="J103" s="4" t="n">
-        <v>0.01545</v>
+        <v>0.0048</v>
       </c>
       <c r="K103" s="3" t="n">
         <f aca="false">SUM(B103:I103)</f>
-        <v>0.488</v>
+        <v>0.032</v>
       </c>
     </row>
     <row r="104" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A104" s="0" t="s">
-        <v>92</v>
+        <v>174</v>
       </c>
       <c r="B104" s="3" t="n">
         <v>0</v>
@@ -8937,7 +8934,7 @@
         <v>0</v>
       </c>
       <c r="E104" s="3" t="n">
-        <v>0</v>
+        <v>0.025</v>
       </c>
       <c r="F104" s="3" t="n">
         <v>0</v>
@@ -8946,17 +8943,17 @@
         <v>0</v>
       </c>
       <c r="H104" s="3" t="n">
-        <v>0.032</v>
+        <v>0</v>
       </c>
       <c r="I104" s="3" t="n">
         <v>0</v>
       </c>
       <c r="J104" s="4" t="n">
-        <v>0.0048</v>
+        <v>0</v>
       </c>
       <c r="K104" s="3" t="n">
         <f aca="false">SUM(B104:I104)</f>
-        <v>0.032</v>
+        <v>0.025</v>
       </c>
     </row>
     <row r="105" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -8973,7 +8970,7 @@
         <v>0</v>
       </c>
       <c r="E105" s="3" t="n">
-        <v>0.024</v>
+        <v>0.05</v>
       </c>
       <c r="F105" s="3" t="n">
         <v>0</v>
@@ -8992,7 +8989,7 @@
       </c>
       <c r="K105" s="3" t="n">
         <f aca="false">SUM(B105:I105)</f>
-        <v>0.024</v>
+        <v>0.05</v>
       </c>
     </row>
     <row r="106" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -9003,13 +9000,13 @@
         <v>0</v>
       </c>
       <c r="C106" s="3" t="n">
-        <v>0</v>
+        <v>0.167</v>
       </c>
       <c r="D106" s="3" t="n">
-        <v>0</v>
+        <v>0.091</v>
       </c>
       <c r="E106" s="3" t="n">
-        <v>0.049</v>
+        <v>0.05</v>
       </c>
       <c r="F106" s="3" t="n">
         <v>0</v>
@@ -9028,7 +9025,7 @@
       </c>
       <c r="K106" s="3" t="n">
         <f aca="false">SUM(B106:I106)</f>
-        <v>0.049</v>
+        <v>0.308</v>
       </c>
     </row>
     <row r="107" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -9039,13 +9036,13 @@
         <v>0</v>
       </c>
       <c r="C107" s="3" t="n">
-        <v>0.158</v>
+        <v>0</v>
       </c>
       <c r="D107" s="3" t="n">
-        <v>0.088</v>
+        <v>0</v>
       </c>
       <c r="E107" s="3" t="n">
-        <v>0.049</v>
+        <v>0.05</v>
       </c>
       <c r="F107" s="3" t="n">
         <v>0</v>
@@ -9064,12 +9061,12 @@
       </c>
       <c r="K107" s="3" t="n">
         <f aca="false">SUM(B107:I107)</f>
-        <v>0.295</v>
+        <v>0.05</v>
       </c>
     </row>
     <row r="108" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A108" s="0" t="s">
-        <v>178</v>
+        <v>99</v>
       </c>
       <c r="B108" s="3" t="n">
         <v>0</v>
@@ -9081,31 +9078,31 @@
         <v>0</v>
       </c>
       <c r="E108" s="3" t="n">
-        <v>0.049</v>
+        <v>0</v>
       </c>
       <c r="F108" s="3" t="n">
         <v>0</v>
       </c>
       <c r="G108" s="3" t="n">
-        <v>0</v>
+        <v>0.023</v>
       </c>
       <c r="H108" s="3" t="n">
-        <v>0</v>
+        <v>0.016</v>
       </c>
       <c r="I108" s="3" t="n">
         <v>0</v>
       </c>
       <c r="J108" s="4" t="n">
-        <v>0</v>
+        <v>0.00447</v>
       </c>
       <c r="K108" s="3" t="n">
         <f aca="false">SUM(B108:I108)</f>
-        <v>0.049</v>
+        <v>0.039</v>
       </c>
     </row>
     <row r="109" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A109" s="0" t="s">
-        <v>99</v>
+        <v>50</v>
       </c>
       <c r="B109" s="3" t="n">
         <v>0</v>
@@ -9123,37 +9120,37 @@
         <v>0</v>
       </c>
       <c r="G109" s="3" t="n">
-        <v>0.023</v>
+        <v>0</v>
       </c>
       <c r="H109" s="3" t="n">
-        <v>0.016</v>
+        <v>0</v>
       </c>
       <c r="I109" s="3" t="n">
-        <v>0</v>
+        <v>0.018</v>
       </c>
       <c r="J109" s="4" t="n">
-        <v>0.00447</v>
+        <v>0.0126</v>
       </c>
       <c r="K109" s="3" t="n">
         <f aca="false">SUM(B109:I109)</f>
-        <v>0.039</v>
+        <v>0.018</v>
       </c>
     </row>
     <row r="110" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A110" s="0" t="s">
-        <v>50</v>
+        <v>178</v>
       </c>
       <c r="B110" s="3" t="n">
-        <v>0</v>
+        <v>0.118</v>
       </c>
       <c r="C110" s="3" t="n">
-        <v>0</v>
+        <v>0.167</v>
       </c>
       <c r="D110" s="3" t="n">
-        <v>0</v>
+        <v>0.091</v>
       </c>
       <c r="E110" s="3" t="n">
-        <v>0</v>
+        <v>0.075</v>
       </c>
       <c r="F110" s="3" t="n">
         <v>0</v>
@@ -9165,34 +9162,34 @@
         <v>0</v>
       </c>
       <c r="I110" s="3" t="n">
-        <v>0.018</v>
+        <v>0</v>
       </c>
       <c r="J110" s="4" t="n">
-        <v>0.0126</v>
+        <v>0</v>
       </c>
       <c r="K110" s="3" t="n">
         <f aca="false">SUM(B110:I110)</f>
-        <v>0.018</v>
+        <v>0.451</v>
       </c>
     </row>
     <row r="111" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A111" s="0" t="s">
-        <v>179</v>
+        <v>123</v>
       </c>
       <c r="B111" s="3" t="n">
-        <v>0.111</v>
+        <v>0</v>
       </c>
       <c r="C111" s="3" t="n">
-        <v>0.158</v>
+        <v>0</v>
       </c>
       <c r="D111" s="3" t="n">
-        <v>0.088</v>
+        <v>0</v>
       </c>
       <c r="E111" s="3" t="n">
-        <v>0.073</v>
+        <v>0</v>
       </c>
       <c r="F111" s="3" t="n">
-        <v>0</v>
+        <v>0.038</v>
       </c>
       <c r="G111" s="3" t="n">
         <v>0</v>
@@ -9204,16 +9201,16 @@
         <v>0</v>
       </c>
       <c r="J111" s="4" t="n">
-        <v>0</v>
+        <v>0.00228</v>
       </c>
       <c r="K111" s="3" t="n">
         <f aca="false">SUM(B111:I111)</f>
-        <v>0.43</v>
+        <v>0.038</v>
       </c>
     </row>
     <row r="112" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A112" s="0" t="s">
-        <v>123</v>
+        <v>108</v>
       </c>
       <c r="B112" s="3" t="n">
         <v>0</v>
@@ -9228,7 +9225,7 @@
         <v>0</v>
       </c>
       <c r="F112" s="3" t="n">
-        <v>0.038</v>
+        <v>0.058</v>
       </c>
       <c r="G112" s="3" t="n">
         <v>0</v>
@@ -9240,22 +9237,22 @@
         <v>0</v>
       </c>
       <c r="J112" s="4" t="n">
-        <v>0.00228</v>
+        <v>0.00348</v>
       </c>
       <c r="K112" s="3" t="n">
         <f aca="false">SUM(B112:I112)</f>
-        <v>0.038</v>
+        <v>0.058</v>
       </c>
     </row>
     <row r="113" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A113" s="0" t="s">
-        <v>108</v>
+        <v>179</v>
       </c>
       <c r="B113" s="3" t="n">
         <v>0</v>
       </c>
       <c r="C113" s="3" t="n">
-        <v>0</v>
+        <v>0.167</v>
       </c>
       <c r="D113" s="3" t="n">
         <v>0</v>
@@ -9264,7 +9261,7 @@
         <v>0</v>
       </c>
       <c r="F113" s="3" t="n">
-        <v>0.058</v>
+        <v>0</v>
       </c>
       <c r="G113" s="3" t="n">
         <v>0</v>
@@ -9276,22 +9273,22 @@
         <v>0</v>
       </c>
       <c r="J113" s="4" t="n">
-        <v>0.00348</v>
+        <v>0</v>
       </c>
       <c r="K113" s="3" t="n">
         <f aca="false">SUM(B113:I113)</f>
-        <v>0.058</v>
+        <v>0.167</v>
       </c>
     </row>
     <row r="114" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A114" s="0" t="s">
-        <v>180</v>
+        <v>104</v>
       </c>
       <c r="B114" s="3" t="n">
         <v>0</v>
       </c>
       <c r="C114" s="3" t="n">
-        <v>0.158</v>
+        <v>0</v>
       </c>
       <c r="D114" s="3" t="n">
         <v>0</v>
@@ -9303,7 +9300,7 @@
         <v>0</v>
       </c>
       <c r="G114" s="3" t="n">
-        <v>0</v>
+        <v>0.047</v>
       </c>
       <c r="H114" s="3" t="n">
         <v>0</v>
@@ -9312,16 +9309,16 @@
         <v>0</v>
       </c>
       <c r="J114" s="4" t="n">
-        <v>0</v>
+        <v>0.00423</v>
       </c>
       <c r="K114" s="3" t="n">
         <f aca="false">SUM(B114:I114)</f>
-        <v>0.158</v>
+        <v>0.047</v>
       </c>
     </row>
     <row r="115" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A115" s="0" t="s">
-        <v>104</v>
+        <v>93</v>
       </c>
       <c r="B115" s="3" t="n">
         <v>0</v>
@@ -9339,25 +9336,25 @@
         <v>0</v>
       </c>
       <c r="G115" s="3" t="n">
-        <v>0.047</v>
+        <v>0</v>
       </c>
       <c r="H115" s="3" t="n">
-        <v>0</v>
+        <v>0.032</v>
       </c>
       <c r="I115" s="3" t="n">
         <v>0</v>
       </c>
       <c r="J115" s="4" t="n">
-        <v>0.00423</v>
+        <v>0.0048</v>
       </c>
       <c r="K115" s="3" t="n">
         <f aca="false">SUM(B115:I115)</f>
-        <v>0.047</v>
+        <v>0.032</v>
       </c>
     </row>
     <row r="116" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A116" s="0" t="s">
-        <v>93</v>
+        <v>41</v>
       </c>
       <c r="B116" s="3" t="n">
         <v>0</v>
@@ -9378,22 +9375,22 @@
         <v>0</v>
       </c>
       <c r="H116" s="3" t="n">
-        <v>0.032</v>
+        <v>0</v>
       </c>
       <c r="I116" s="3" t="n">
-        <v>0</v>
+        <v>0.036</v>
       </c>
       <c r="J116" s="4" t="n">
-        <v>0.0048</v>
+        <v>0.0252</v>
       </c>
       <c r="K116" s="3" t="n">
         <f aca="false">SUM(B116:I116)</f>
-        <v>0.032</v>
+        <v>0.036</v>
       </c>
     </row>
     <row r="117" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A117" s="0" t="s">
-        <v>41</v>
+        <v>80</v>
       </c>
       <c r="B117" s="3" t="n">
         <v>0</v>
@@ -9411,25 +9408,25 @@
         <v>0</v>
       </c>
       <c r="G117" s="3" t="n">
-        <v>0</v>
+        <v>0.07</v>
       </c>
       <c r="H117" s="3" t="n">
         <v>0</v>
       </c>
       <c r="I117" s="3" t="n">
-        <v>0.036</v>
+        <v>0</v>
       </c>
       <c r="J117" s="4" t="n">
-        <v>0.0252</v>
+        <v>0.0063</v>
       </c>
       <c r="K117" s="3" t="n">
         <f aca="false">SUM(B117:I117)</f>
-        <v>0.036</v>
+        <v>0.07</v>
       </c>
     </row>
     <row r="118" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A118" s="0" t="s">
-        <v>80</v>
+        <v>77</v>
       </c>
       <c r="B118" s="3" t="n">
         <v>0</v>
@@ -9447,25 +9444,25 @@
         <v>0</v>
       </c>
       <c r="G118" s="3" t="n">
-        <v>0.07</v>
+        <v>0</v>
       </c>
       <c r="H118" s="3" t="n">
-        <v>0</v>
+        <v>0.048</v>
       </c>
       <c r="I118" s="3" t="n">
         <v>0</v>
       </c>
       <c r="J118" s="4" t="n">
-        <v>0.0063</v>
+        <v>0.0072</v>
       </c>
       <c r="K118" s="3" t="n">
         <f aca="false">SUM(B118:I118)</f>
-        <v>0.07</v>
+        <v>0.048</v>
       </c>
     </row>
     <row r="119" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A119" s="0" t="s">
-        <v>77</v>
+        <v>42</v>
       </c>
       <c r="B119" s="3" t="n">
         <v>0</v>
@@ -9474,7 +9471,7 @@
         <v>0</v>
       </c>
       <c r="D119" s="3" t="n">
-        <v>0</v>
+        <v>0.242</v>
       </c>
       <c r="E119" s="3" t="n">
         <v>0</v>
@@ -9483,25 +9480,25 @@
         <v>0</v>
       </c>
       <c r="G119" s="3" t="n">
-        <v>0</v>
+        <v>0.047</v>
       </c>
       <c r="H119" s="3" t="n">
-        <v>0.048</v>
+        <v>0.032</v>
       </c>
       <c r="I119" s="3" t="n">
-        <v>0</v>
+        <v>0.036</v>
       </c>
       <c r="J119" s="4" t="n">
-        <v>0.0072</v>
+        <v>0.03423</v>
       </c>
       <c r="K119" s="3" t="n">
         <f aca="false">SUM(B119:I119)</f>
-        <v>0.048</v>
+        <v>0.357</v>
       </c>
     </row>
     <row r="120" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A120" s="0" t="s">
-        <v>42</v>
+        <v>117</v>
       </c>
       <c r="B120" s="3" t="n">
         <v>0</v>
@@ -9510,46 +9507,46 @@
         <v>0</v>
       </c>
       <c r="D120" s="3" t="n">
-        <v>0.235</v>
+        <v>0</v>
       </c>
       <c r="E120" s="3" t="n">
-        <v>0</v>
+        <v>0.075</v>
       </c>
       <c r="F120" s="3" t="n">
         <v>0</v>
       </c>
       <c r="G120" s="3" t="n">
-        <v>0.047</v>
+        <v>0</v>
       </c>
       <c r="H120" s="3" t="n">
-        <v>0.032</v>
+        <v>0.016</v>
       </c>
       <c r="I120" s="3" t="n">
-        <v>0.036</v>
+        <v>0</v>
       </c>
       <c r="J120" s="4" t="n">
-        <v>0.03423</v>
+        <v>0.0024</v>
       </c>
       <c r="K120" s="3" t="n">
         <f aca="false">SUM(B120:I120)</f>
-        <v>0.35</v>
+        <v>0.091</v>
       </c>
     </row>
     <row r="121" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A121" s="0" t="s">
-        <v>117</v>
+        <v>180</v>
       </c>
       <c r="B121" s="3" t="n">
         <v>0</v>
       </c>
       <c r="C121" s="3" t="n">
-        <v>0</v>
+        <v>0.167</v>
       </c>
       <c r="D121" s="3" t="n">
         <v>0</v>
       </c>
       <c r="E121" s="3" t="n">
-        <v>0.073</v>
+        <v>0</v>
       </c>
       <c r="F121" s="3" t="n">
         <v>0</v>
@@ -9558,40 +9555,40 @@
         <v>0</v>
       </c>
       <c r="H121" s="3" t="n">
-        <v>0.016</v>
+        <v>0</v>
       </c>
       <c r="I121" s="3" t="n">
         <v>0</v>
       </c>
       <c r="J121" s="4" t="n">
-        <v>0.0024</v>
+        <v>0</v>
       </c>
       <c r="K121" s="3" t="n">
         <f aca="false">SUM(B121:I121)</f>
-        <v>0.089</v>
+        <v>0.167</v>
       </c>
     </row>
     <row r="122" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A122" s="0" t="s">
-        <v>181</v>
+        <v>64</v>
       </c>
       <c r="B122" s="3" t="n">
         <v>0</v>
       </c>
       <c r="C122" s="3" t="n">
-        <v>0.158</v>
+        <v>0</v>
       </c>
       <c r="D122" s="3" t="n">
-        <v>0</v>
+        <v>0.091</v>
       </c>
       <c r="E122" s="3" t="n">
         <v>0</v>
       </c>
       <c r="F122" s="3" t="n">
-        <v>0</v>
+        <v>0.154</v>
       </c>
       <c r="G122" s="3" t="n">
-        <v>0</v>
+        <v>0.07</v>
       </c>
       <c r="H122" s="3" t="n">
         <v>0</v>
@@ -9600,16 +9597,16 @@
         <v>0</v>
       </c>
       <c r="J122" s="4" t="n">
-        <v>0</v>
+        <v>0.01554</v>
       </c>
       <c r="K122" s="3" t="n">
         <f aca="false">SUM(B122:I122)</f>
-        <v>0.158</v>
+        <v>0.315</v>
       </c>
     </row>
     <row r="123" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A123" s="0" t="s">
-        <v>64</v>
+        <v>78</v>
       </c>
       <c r="B123" s="3" t="n">
         <v>0</v>
@@ -9618,34 +9615,34 @@
         <v>0</v>
       </c>
       <c r="D123" s="3" t="n">
-        <v>0.088</v>
+        <v>0.03</v>
       </c>
       <c r="E123" s="3" t="n">
         <v>0</v>
       </c>
       <c r="F123" s="3" t="n">
-        <v>0.154</v>
+        <v>0</v>
       </c>
       <c r="G123" s="3" t="n">
-        <v>0.07</v>
+        <v>0</v>
       </c>
       <c r="H123" s="3" t="n">
-        <v>0</v>
+        <v>0.048</v>
       </c>
       <c r="I123" s="3" t="n">
         <v>0</v>
       </c>
       <c r="J123" s="4" t="n">
-        <v>0.01554</v>
+        <v>0.0072</v>
       </c>
       <c r="K123" s="3" t="n">
         <f aca="false">SUM(B123:I123)</f>
-        <v>0.312</v>
+        <v>0.078</v>
       </c>
     </row>
     <row r="124" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A124" s="0" t="s">
-        <v>78</v>
+        <v>109</v>
       </c>
       <c r="B124" s="3" t="n">
         <v>0</v>
@@ -9654,34 +9651,34 @@
         <v>0</v>
       </c>
       <c r="D124" s="3" t="n">
-        <v>0.029</v>
+        <v>0</v>
       </c>
       <c r="E124" s="3" t="n">
         <v>0</v>
       </c>
       <c r="F124" s="3" t="n">
-        <v>0</v>
+        <v>0.058</v>
       </c>
       <c r="G124" s="3" t="n">
         <v>0</v>
       </c>
       <c r="H124" s="3" t="n">
-        <v>0.048</v>
+        <v>0</v>
       </c>
       <c r="I124" s="3" t="n">
         <v>0</v>
       </c>
       <c r="J124" s="4" t="n">
-        <v>0.0072</v>
+        <v>0.00348</v>
       </c>
       <c r="K124" s="3" t="n">
         <f aca="false">SUM(B124:I124)</f>
-        <v>0.077</v>
+        <v>0.058</v>
       </c>
     </row>
     <row r="125" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A125" s="0" t="s">
-        <v>109</v>
+        <v>43</v>
       </c>
       <c r="B125" s="3" t="n">
         <v>0</v>
@@ -9696,7 +9693,7 @@
         <v>0</v>
       </c>
       <c r="F125" s="3" t="n">
-        <v>0.058</v>
+        <v>0</v>
       </c>
       <c r="G125" s="3" t="n">
         <v>0</v>
@@ -9705,19 +9702,19 @@
         <v>0</v>
       </c>
       <c r="I125" s="3" t="n">
-        <v>0</v>
+        <v>0.036</v>
       </c>
       <c r="J125" s="4" t="n">
-        <v>0.00348</v>
+        <v>0.0252</v>
       </c>
       <c r="K125" s="3" t="n">
         <f aca="false">SUM(B125:I125)</f>
-        <v>0.058</v>
+        <v>0.036</v>
       </c>
     </row>
     <row r="126" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A126" s="0" t="s">
-        <v>43</v>
+        <v>94</v>
       </c>
       <c r="B126" s="3" t="n">
         <v>0</v>
@@ -9738,28 +9735,28 @@
         <v>0</v>
       </c>
       <c r="H126" s="3" t="n">
-        <v>0</v>
+        <v>0.032</v>
       </c>
       <c r="I126" s="3" t="n">
-        <v>0.036</v>
+        <v>0</v>
       </c>
       <c r="J126" s="4" t="n">
-        <v>0.0252</v>
+        <v>0.0048</v>
       </c>
       <c r="K126" s="3" t="n">
         <f aca="false">SUM(B126:I126)</f>
-        <v>0.036</v>
+        <v>0.032</v>
       </c>
     </row>
     <row r="127" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A127" s="0" t="s">
-        <v>94</v>
+        <v>181</v>
       </c>
       <c r="B127" s="3" t="n">
         <v>0</v>
       </c>
       <c r="C127" s="3" t="n">
-        <v>0</v>
+        <v>0.056</v>
       </c>
       <c r="D127" s="3" t="n">
         <v>0</v>
@@ -9774,58 +9771,58 @@
         <v>0</v>
       </c>
       <c r="H127" s="3" t="n">
-        <v>0.032</v>
+        <v>0</v>
       </c>
       <c r="I127" s="3" t="n">
         <v>0</v>
       </c>
       <c r="J127" s="4" t="n">
-        <v>0.0048</v>
+        <v>0</v>
       </c>
       <c r="K127" s="3" t="n">
         <f aca="false">SUM(B127:I127)</f>
-        <v>0.032</v>
+        <v>0.056</v>
       </c>
     </row>
     <row r="128" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A128" s="0" t="s">
-        <v>182</v>
+        <v>60</v>
       </c>
       <c r="B128" s="3" t="n">
         <v>0</v>
       </c>
       <c r="C128" s="3" t="n">
-        <v>0.053</v>
+        <v>0</v>
       </c>
       <c r="D128" s="3" t="n">
         <v>0</v>
       </c>
       <c r="E128" s="3" t="n">
-        <v>0</v>
+        <v>0.05</v>
       </c>
       <c r="F128" s="3" t="n">
-        <v>0</v>
+        <v>0.135</v>
       </c>
       <c r="G128" s="3" t="n">
-        <v>0</v>
+        <v>0.047</v>
       </c>
       <c r="H128" s="3" t="n">
-        <v>0</v>
+        <v>0.063</v>
       </c>
       <c r="I128" s="3" t="n">
         <v>0</v>
       </c>
       <c r="J128" s="4" t="n">
-        <v>0</v>
+        <v>0.02178</v>
       </c>
       <c r="K128" s="3" t="n">
         <f aca="false">SUM(B128:I128)</f>
-        <v>0.053</v>
+        <v>0.295</v>
       </c>
     </row>
     <row r="129" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A129" s="0" t="s">
-        <v>60</v>
+        <v>182</v>
       </c>
       <c r="B129" s="3" t="n">
         <v>0</v>
@@ -9834,34 +9831,34 @@
         <v>0</v>
       </c>
       <c r="D129" s="3" t="n">
-        <v>0</v>
+        <v>0.061</v>
       </c>
       <c r="E129" s="3" t="n">
-        <v>0.049</v>
+        <v>0</v>
       </c>
       <c r="F129" s="3" t="n">
-        <v>0.135</v>
+        <v>0</v>
       </c>
       <c r="G129" s="3" t="n">
-        <v>0.047</v>
+        <v>0</v>
       </c>
       <c r="H129" s="3" t="n">
-        <v>0.063</v>
+        <v>0</v>
       </c>
       <c r="I129" s="3" t="n">
         <v>0</v>
       </c>
       <c r="J129" s="4" t="n">
-        <v>0.02178</v>
+        <v>0</v>
       </c>
       <c r="K129" s="3" t="n">
         <f aca="false">SUM(B129:I129)</f>
-        <v>0.294</v>
+        <v>0.061</v>
       </c>
     </row>
     <row r="130" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A130" s="0" t="s">
-        <v>183</v>
+        <v>67</v>
       </c>
       <c r="B130" s="3" t="n">
         <v>0</v>
@@ -9870,7 +9867,7 @@
         <v>0</v>
       </c>
       <c r="D130" s="3" t="n">
-        <v>0.059</v>
+        <v>0</v>
       </c>
       <c r="E130" s="3" t="n">
         <v>0</v>
@@ -9879,25 +9876,25 @@
         <v>0</v>
       </c>
       <c r="G130" s="3" t="n">
-        <v>0</v>
+        <v>0.07</v>
       </c>
       <c r="H130" s="3" t="n">
-        <v>0</v>
+        <v>0.032</v>
       </c>
       <c r="I130" s="3" t="n">
         <v>0</v>
       </c>
       <c r="J130" s="4" t="n">
-        <v>0</v>
+        <v>0.0111</v>
       </c>
       <c r="K130" s="3" t="n">
         <f aca="false">SUM(B130:I130)</f>
-        <v>0.059</v>
+        <v>0.102</v>
       </c>
     </row>
     <row r="131" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A131" s="0" t="s">
-        <v>67</v>
+        <v>16</v>
       </c>
       <c r="B131" s="3" t="n">
         <v>0</v>
@@ -9909,31 +9906,31 @@
         <v>0</v>
       </c>
       <c r="E131" s="3" t="n">
-        <v>0</v>
+        <v>0.05</v>
       </c>
       <c r="F131" s="3" t="n">
-        <v>0</v>
+        <v>0.154</v>
       </c>
       <c r="G131" s="3" t="n">
-        <v>0.07</v>
+        <v>0.14</v>
       </c>
       <c r="H131" s="3" t="n">
-        <v>0.032</v>
+        <v>0.143</v>
       </c>
       <c r="I131" s="3" t="n">
-        <v>0</v>
+        <v>0.091</v>
       </c>
       <c r="J131" s="4" t="n">
-        <v>0.0111</v>
+        <v>0.10699</v>
       </c>
       <c r="K131" s="3" t="n">
         <f aca="false">SUM(B131:I131)</f>
-        <v>0.102</v>
+        <v>0.578</v>
       </c>
     </row>
     <row r="132" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A132" s="0" t="s">
-        <v>16</v>
+        <v>118</v>
       </c>
       <c r="B132" s="3" t="n">
         <v>0</v>
@@ -9945,31 +9942,31 @@
         <v>0</v>
       </c>
       <c r="E132" s="3" t="n">
-        <v>0.049</v>
+        <v>0</v>
       </c>
       <c r="F132" s="3" t="n">
-        <v>0.154</v>
+        <v>0</v>
       </c>
       <c r="G132" s="3" t="n">
-        <v>0.14</v>
+        <v>0</v>
       </c>
       <c r="H132" s="3" t="n">
-        <v>0.143</v>
+        <v>0.016</v>
       </c>
       <c r="I132" s="3" t="n">
-        <v>0.091</v>
+        <v>0</v>
       </c>
       <c r="J132" s="4" t="n">
-        <v>0.10699</v>
+        <v>0.0024</v>
       </c>
       <c r="K132" s="3" t="n">
         <f aca="false">SUM(B132:I132)</f>
-        <v>0.577</v>
+        <v>0.016</v>
       </c>
     </row>
     <row r="133" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A133" s="0" t="s">
-        <v>118</v>
+        <v>183</v>
       </c>
       <c r="B133" s="3" t="n">
         <v>0</v>
@@ -9981,7 +9978,7 @@
         <v>0</v>
       </c>
       <c r="E133" s="3" t="n">
-        <v>0</v>
+        <v>0.075</v>
       </c>
       <c r="F133" s="3" t="n">
         <v>0</v>
@@ -9990,22 +9987,22 @@
         <v>0</v>
       </c>
       <c r="H133" s="3" t="n">
-        <v>0.016</v>
+        <v>0</v>
       </c>
       <c r="I133" s="3" t="n">
         <v>0</v>
       </c>
       <c r="J133" s="4" t="n">
-        <v>0.0024</v>
+        <v>0</v>
       </c>
       <c r="K133" s="3" t="n">
         <f aca="false">SUM(B133:I133)</f>
-        <v>0.016</v>
+        <v>0.075</v>
       </c>
     </row>
     <row r="134" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A134" s="0" t="s">
-        <v>184</v>
+        <v>70</v>
       </c>
       <c r="B134" s="3" t="n">
         <v>0</v>
@@ -10014,34 +10011,34 @@
         <v>0</v>
       </c>
       <c r="D134" s="3" t="n">
-        <v>0</v>
+        <v>0.152</v>
       </c>
       <c r="E134" s="3" t="n">
-        <v>0.073</v>
+        <v>0.05</v>
       </c>
       <c r="F134" s="3" t="n">
         <v>0</v>
       </c>
       <c r="G134" s="3" t="n">
-        <v>0</v>
+        <v>0.023</v>
       </c>
       <c r="H134" s="3" t="n">
-        <v>0</v>
+        <v>0.048</v>
       </c>
       <c r="I134" s="3" t="n">
         <v>0</v>
       </c>
       <c r="J134" s="4" t="n">
-        <v>0</v>
+        <v>0.00927</v>
       </c>
       <c r="K134" s="3" t="n">
         <f aca="false">SUM(B134:I134)</f>
-        <v>0.073</v>
+        <v>0.273</v>
       </c>
     </row>
     <row r="135" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A135" s="0" t="s">
-        <v>70</v>
+        <v>25</v>
       </c>
       <c r="B135" s="3" t="n">
         <v>0</v>
@@ -10050,85 +10047,85 @@
         <v>0</v>
       </c>
       <c r="D135" s="3" t="n">
-        <v>0.147</v>
+        <v>0</v>
       </c>
       <c r="E135" s="3" t="n">
-        <v>0.049</v>
+        <v>0</v>
       </c>
       <c r="F135" s="3" t="n">
         <v>0</v>
       </c>
       <c r="G135" s="3" t="n">
-        <v>0.023</v>
+        <v>0</v>
       </c>
       <c r="H135" s="3" t="n">
-        <v>0.048</v>
+        <v>0.032</v>
       </c>
       <c r="I135" s="3" t="n">
-        <v>0</v>
+        <v>0.055</v>
       </c>
       <c r="J135" s="4" t="n">
-        <v>0.00927</v>
+        <v>0.0433</v>
       </c>
       <c r="K135" s="3" t="n">
         <f aca="false">SUM(B135:I135)</f>
-        <v>0.267</v>
+        <v>0.087</v>
       </c>
     </row>
     <row r="136" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A136" s="0" t="s">
-        <v>25</v>
+        <v>12</v>
       </c>
       <c r="B136" s="3" t="n">
-        <v>0</v>
+        <v>0.529</v>
       </c>
       <c r="C136" s="3" t="n">
-        <v>0</v>
+        <v>0.056</v>
       </c>
       <c r="D136" s="3" t="n">
-        <v>0</v>
+        <v>0.091</v>
       </c>
       <c r="E136" s="3" t="n">
-        <v>0</v>
+        <v>0.15</v>
       </c>
       <c r="F136" s="3" t="n">
-        <v>0</v>
+        <v>0.115</v>
       </c>
       <c r="G136" s="3" t="n">
-        <v>0</v>
+        <v>0.023</v>
       </c>
       <c r="H136" s="3" t="n">
-        <v>0.032</v>
+        <v>0</v>
       </c>
       <c r="I136" s="3" t="n">
-        <v>0.055</v>
+        <v>0.127</v>
       </c>
       <c r="J136" s="4" t="n">
-        <v>0.0433</v>
+        <v>0.09787</v>
       </c>
       <c r="K136" s="3" t="n">
         <f aca="false">SUM(B136:I136)</f>
-        <v>0.087</v>
+        <v>1.091</v>
       </c>
     </row>
     <row r="137" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A137" s="0" t="s">
-        <v>12</v>
+        <v>128</v>
       </c>
       <c r="B137" s="3" t="n">
-        <v>0.5</v>
+        <v>0</v>
       </c>
       <c r="C137" s="3" t="n">
-        <v>0.053</v>
+        <v>0</v>
       </c>
       <c r="D137" s="3" t="n">
-        <v>0.088</v>
+        <v>0</v>
       </c>
       <c r="E137" s="3" t="n">
-        <v>0.146</v>
+        <v>0</v>
       </c>
       <c r="F137" s="3" t="n">
-        <v>0.115</v>
+        <v>0</v>
       </c>
       <c r="G137" s="3" t="n">
         <v>0.023</v>
@@ -10137,25 +10134,25 @@
         <v>0</v>
       </c>
       <c r="I137" s="3" t="n">
-        <v>0.127</v>
+        <v>0</v>
       </c>
       <c r="J137" s="4" t="n">
-        <v>0.09787</v>
+        <v>0.00207</v>
       </c>
       <c r="K137" s="3" t="n">
         <f aca="false">SUM(B137:I137)</f>
-        <v>1.052</v>
+        <v>0.023</v>
       </c>
     </row>
     <row r="138" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A138" s="0" t="s">
-        <v>128</v>
+        <v>51</v>
       </c>
       <c r="B138" s="3" t="n">
         <v>0</v>
       </c>
       <c r="C138" s="3" t="n">
-        <v>0</v>
+        <v>0.111</v>
       </c>
       <c r="D138" s="3" t="n">
         <v>0</v>
@@ -10167,31 +10164,31 @@
         <v>0</v>
       </c>
       <c r="G138" s="3" t="n">
-        <v>0.023</v>
+        <v>0</v>
       </c>
       <c r="H138" s="3" t="n">
-        <v>0</v>
+        <v>0.048</v>
       </c>
       <c r="I138" s="3" t="n">
-        <v>0</v>
+        <v>0.018</v>
       </c>
       <c r="J138" s="4" t="n">
-        <v>0.00207</v>
+        <v>0.0198</v>
       </c>
       <c r="K138" s="3" t="n">
         <f aca="false">SUM(B138:I138)</f>
-        <v>0.023</v>
+        <v>0.177</v>
       </c>
     </row>
     <row r="139" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A139" s="0" t="s">
-        <v>51</v>
+        <v>124</v>
       </c>
       <c r="B139" s="3" t="n">
         <v>0</v>
       </c>
       <c r="C139" s="3" t="n">
-        <v>0.105</v>
+        <v>0</v>
       </c>
       <c r="D139" s="3" t="n">
         <v>0</v>
@@ -10200,28 +10197,28 @@
         <v>0</v>
       </c>
       <c r="F139" s="3" t="n">
-        <v>0</v>
+        <v>0.038</v>
       </c>
       <c r="G139" s="3" t="n">
         <v>0</v>
       </c>
       <c r="H139" s="3" t="n">
-        <v>0.048</v>
+        <v>0</v>
       </c>
       <c r="I139" s="3" t="n">
-        <v>0.018</v>
+        <v>0</v>
       </c>
       <c r="J139" s="4" t="n">
-        <v>0.0198</v>
+        <v>0.00228</v>
       </c>
       <c r="K139" s="3" t="n">
         <f aca="false">SUM(B139:I139)</f>
-        <v>0.171</v>
+        <v>0.038</v>
       </c>
     </row>
     <row r="140" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A140" s="0" t="s">
-        <v>124</v>
+        <v>110</v>
       </c>
       <c r="B140" s="3" t="n">
         <v>0</v>
@@ -10236,7 +10233,7 @@
         <v>0</v>
       </c>
       <c r="F140" s="3" t="n">
-        <v>0.038</v>
+        <v>0.058</v>
       </c>
       <c r="G140" s="3" t="n">
         <v>0</v>
@@ -10248,16 +10245,16 @@
         <v>0</v>
       </c>
       <c r="J140" s="4" t="n">
-        <v>0.00228</v>
+        <v>0.00348</v>
       </c>
       <c r="K140" s="3" t="n">
         <f aca="false">SUM(B140:I140)</f>
-        <v>0.038</v>
+        <v>0.058</v>
       </c>
     </row>
     <row r="141" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A141" s="0" t="s">
-        <v>110</v>
+        <v>95</v>
       </c>
       <c r="B141" s="3" t="n">
         <v>0</v>
@@ -10272,28 +10269,28 @@
         <v>0</v>
       </c>
       <c r="F141" s="3" t="n">
-        <v>0.058</v>
+        <v>0</v>
       </c>
       <c r="G141" s="3" t="n">
         <v>0</v>
       </c>
       <c r="H141" s="3" t="n">
-        <v>0</v>
+        <v>0.032</v>
       </c>
       <c r="I141" s="3" t="n">
         <v>0</v>
       </c>
       <c r="J141" s="4" t="n">
-        <v>0.00348</v>
+        <v>0.0048</v>
       </c>
       <c r="K141" s="3" t="n">
         <f aca="false">SUM(B141:I141)</f>
-        <v>0.058</v>
+        <v>0.032</v>
       </c>
     </row>
     <row r="142" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A142" s="0" t="s">
-        <v>95</v>
+        <v>52</v>
       </c>
       <c r="B142" s="3" t="n">
         <v>0</v>
@@ -10308,28 +10305,28 @@
         <v>0</v>
       </c>
       <c r="F142" s="3" t="n">
-        <v>0</v>
+        <v>0.096</v>
       </c>
       <c r="G142" s="3" t="n">
-        <v>0</v>
+        <v>0.047</v>
       </c>
       <c r="H142" s="3" t="n">
         <v>0.032</v>
       </c>
       <c r="I142" s="3" t="n">
-        <v>0</v>
+        <v>0.018</v>
       </c>
       <c r="J142" s="4" t="n">
-        <v>0.0048</v>
+        <v>0.02739</v>
       </c>
       <c r="K142" s="3" t="n">
         <f aca="false">SUM(B142:I142)</f>
-        <v>0.032</v>
+        <v>0.193</v>
       </c>
     </row>
     <row r="143" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A143" s="0" t="s">
-        <v>52</v>
+        <v>184</v>
       </c>
       <c r="B143" s="3" t="n">
         <v>0</v>
@@ -10338,34 +10335,34 @@
         <v>0</v>
       </c>
       <c r="D143" s="3" t="n">
-        <v>0</v>
+        <v>0.061</v>
       </c>
       <c r="E143" s="3" t="n">
         <v>0</v>
       </c>
       <c r="F143" s="3" t="n">
-        <v>0.096</v>
+        <v>0</v>
       </c>
       <c r="G143" s="3" t="n">
-        <v>0.047</v>
+        <v>0</v>
       </c>
       <c r="H143" s="3" t="n">
-        <v>0.032</v>
+        <v>0</v>
       </c>
       <c r="I143" s="3" t="n">
-        <v>0.018</v>
+        <v>0</v>
       </c>
       <c r="J143" s="4" t="n">
-        <v>0.02739</v>
+        <v>0</v>
       </c>
       <c r="K143" s="3" t="n">
         <f aca="false">SUM(B143:I143)</f>
-        <v>0.193</v>
+        <v>0.061</v>
       </c>
     </row>
     <row r="144" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A144" s="0" t="s">
-        <v>185</v>
+        <v>26</v>
       </c>
       <c r="B144" s="3" t="n">
         <v>0</v>
@@ -10374,34 +10371,34 @@
         <v>0</v>
       </c>
       <c r="D144" s="3" t="n">
-        <v>0.059</v>
+        <v>0</v>
       </c>
       <c r="E144" s="3" t="n">
         <v>0</v>
       </c>
       <c r="F144" s="3" t="n">
-        <v>0</v>
+        <v>0.096</v>
       </c>
       <c r="G144" s="3" t="n">
         <v>0</v>
       </c>
       <c r="H144" s="3" t="n">
-        <v>0</v>
+        <v>0.095</v>
       </c>
       <c r="I144" s="3" t="n">
-        <v>0</v>
+        <v>0.055</v>
       </c>
       <c r="J144" s="4" t="n">
-        <v>0</v>
+        <v>0.05851</v>
       </c>
       <c r="K144" s="3" t="n">
         <f aca="false">SUM(B144:I144)</f>
-        <v>0.059</v>
+        <v>0.246</v>
       </c>
     </row>
     <row r="145" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A145" s="0" t="s">
-        <v>26</v>
+        <v>185</v>
       </c>
       <c r="B145" s="3" t="n">
         <v>0</v>
@@ -10413,31 +10410,31 @@
         <v>0</v>
       </c>
       <c r="E145" s="3" t="n">
-        <v>0</v>
+        <v>0.05</v>
       </c>
       <c r="F145" s="3" t="n">
-        <v>0.096</v>
+        <v>0</v>
       </c>
       <c r="G145" s="3" t="n">
         <v>0</v>
       </c>
       <c r="H145" s="3" t="n">
-        <v>0.095</v>
+        <v>0</v>
       </c>
       <c r="I145" s="3" t="n">
-        <v>0.055</v>
+        <v>0</v>
       </c>
       <c r="J145" s="4" t="n">
-        <v>0.05851</v>
+        <v>0</v>
       </c>
       <c r="K145" s="3" t="n">
         <f aca="false">SUM(B145:I145)</f>
-        <v>0.246</v>
+        <v>0.05</v>
       </c>
     </row>
     <row r="146" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A146" s="0" t="s">
-        <v>186</v>
+        <v>119</v>
       </c>
       <c r="B146" s="3" t="n">
         <v>0</v>
@@ -10449,7 +10446,7 @@
         <v>0</v>
       </c>
       <c r="E146" s="3" t="n">
-        <v>0.049</v>
+        <v>0</v>
       </c>
       <c r="F146" s="3" t="n">
         <v>0</v>
@@ -10458,22 +10455,22 @@
         <v>0</v>
       </c>
       <c r="H146" s="3" t="n">
-        <v>0</v>
+        <v>0.016</v>
       </c>
       <c r="I146" s="3" t="n">
         <v>0</v>
       </c>
       <c r="J146" s="4" t="n">
-        <v>0</v>
+        <v>0.0024</v>
       </c>
       <c r="K146" s="3" t="n">
         <f aca="false">SUM(B146:I146)</f>
-        <v>0.049</v>
+        <v>0.016</v>
       </c>
     </row>
     <row r="147" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A147" s="0" t="s">
-        <v>119</v>
+        <v>186</v>
       </c>
       <c r="B147" s="3" t="n">
         <v>0</v>
@@ -10482,10 +10479,10 @@
         <v>0</v>
       </c>
       <c r="D147" s="3" t="n">
-        <v>0</v>
+        <v>0.091</v>
       </c>
       <c r="E147" s="3" t="n">
-        <v>0</v>
+        <v>0.025</v>
       </c>
       <c r="F147" s="3" t="n">
         <v>0</v>
@@ -10494,22 +10491,22 @@
         <v>0</v>
       </c>
       <c r="H147" s="3" t="n">
-        <v>0.016</v>
+        <v>0</v>
       </c>
       <c r="I147" s="3" t="n">
         <v>0</v>
       </c>
       <c r="J147" s="4" t="n">
-        <v>0.0024</v>
+        <v>0</v>
       </c>
       <c r="K147" s="3" t="n">
         <f aca="false">SUM(B147:I147)</f>
-        <v>0.016</v>
+        <v>0.116</v>
       </c>
     </row>
     <row r="148" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A148" s="0" t="s">
-        <v>187</v>
+        <v>53</v>
       </c>
       <c r="B148" s="3" t="n">
         <v>0</v>
@@ -10518,10 +10515,10 @@
         <v>0</v>
       </c>
       <c r="D148" s="3" t="n">
-        <v>0.088</v>
+        <v>0</v>
       </c>
       <c r="E148" s="3" t="n">
-        <v>0.024</v>
+        <v>0</v>
       </c>
       <c r="F148" s="3" t="n">
         <v>0</v>
@@ -10533,19 +10530,19 @@
         <v>0</v>
       </c>
       <c r="I148" s="3" t="n">
-        <v>0</v>
+        <v>0.018</v>
       </c>
       <c r="J148" s="4" t="n">
-        <v>0</v>
+        <v>0.0126</v>
       </c>
       <c r="K148" s="3" t="n">
         <f aca="false">SUM(B148:I148)</f>
-        <v>0.112</v>
+        <v>0.018</v>
       </c>
     </row>
     <row r="149" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A149" s="0" t="s">
-        <v>53</v>
+        <v>96</v>
       </c>
       <c r="B149" s="3" t="n">
         <v>0</v>
@@ -10566,28 +10563,28 @@
         <v>0</v>
       </c>
       <c r="H149" s="3" t="n">
-        <v>0</v>
+        <v>0.032</v>
       </c>
       <c r="I149" s="3" t="n">
-        <v>0.018</v>
+        <v>0</v>
       </c>
       <c r="J149" s="4" t="n">
-        <v>0.0126</v>
+        <v>0.0048</v>
       </c>
       <c r="K149" s="3" t="n">
         <f aca="false">SUM(B149:I149)</f>
-        <v>0.018</v>
+        <v>0.032</v>
       </c>
     </row>
     <row r="150" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A150" s="0" t="s">
-        <v>96</v>
+        <v>44</v>
       </c>
       <c r="B150" s="3" t="n">
         <v>0</v>
       </c>
       <c r="C150" s="3" t="n">
-        <v>0</v>
+        <v>0.111</v>
       </c>
       <c r="D150" s="3" t="n">
         <v>0</v>
@@ -10599,61 +10596,61 @@
         <v>0</v>
       </c>
       <c r="G150" s="3" t="n">
-        <v>0</v>
+        <v>0.023</v>
       </c>
       <c r="H150" s="3" t="n">
-        <v>0.032</v>
+        <v>0</v>
       </c>
       <c r="I150" s="3" t="n">
-        <v>0</v>
+        <v>0.036</v>
       </c>
       <c r="J150" s="4" t="n">
-        <v>0.0048</v>
+        <v>0.02727</v>
       </c>
       <c r="K150" s="3" t="n">
         <f aca="false">SUM(B150:I150)</f>
-        <v>0.032</v>
+        <v>0.17</v>
       </c>
     </row>
     <row r="151" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A151" s="0" t="s">
-        <v>44</v>
+        <v>27</v>
       </c>
       <c r="B151" s="3" t="n">
         <v>0</v>
       </c>
       <c r="C151" s="3" t="n">
-        <v>0.105</v>
+        <v>0</v>
       </c>
       <c r="D151" s="3" t="n">
         <v>0</v>
       </c>
       <c r="E151" s="3" t="n">
-        <v>0</v>
+        <v>0.075</v>
       </c>
       <c r="F151" s="3" t="n">
-        <v>0</v>
+        <v>0.058</v>
       </c>
       <c r="G151" s="3" t="n">
         <v>0.023</v>
       </c>
       <c r="H151" s="3" t="n">
-        <v>0</v>
+        <v>0.048</v>
       </c>
       <c r="I151" s="3" t="n">
-        <v>0.036</v>
+        <v>0.055</v>
       </c>
       <c r="J151" s="4" t="n">
-        <v>0.02727</v>
+        <v>0.05125</v>
       </c>
       <c r="K151" s="3" t="n">
         <f aca="false">SUM(B151:I151)</f>
-        <v>0.164</v>
+        <v>0.259</v>
       </c>
     </row>
     <row r="152" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A152" s="0" t="s">
-        <v>27</v>
+        <v>111</v>
       </c>
       <c r="B152" s="3" t="n">
         <v>0</v>
@@ -10665,46 +10662,46 @@
         <v>0</v>
       </c>
       <c r="E152" s="3" t="n">
-        <v>0.073</v>
+        <v>0</v>
       </c>
       <c r="F152" s="3" t="n">
         <v>0.058</v>
       </c>
       <c r="G152" s="3" t="n">
-        <v>0.023</v>
+        <v>0</v>
       </c>
       <c r="H152" s="3" t="n">
-        <v>0.048</v>
+        <v>0</v>
       </c>
       <c r="I152" s="3" t="n">
-        <v>0.055</v>
+        <v>0</v>
       </c>
       <c r="J152" s="4" t="n">
-        <v>0.05125</v>
+        <v>0.00348</v>
       </c>
       <c r="K152" s="3" t="n">
         <f aca="false">SUM(B152:I152)</f>
-        <v>0.257</v>
+        <v>0.058</v>
       </c>
     </row>
     <row r="153" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A153" s="0" t="s">
-        <v>111</v>
+        <v>125</v>
       </c>
       <c r="B153" s="3" t="n">
-        <v>0</v>
+        <v>0.176</v>
       </c>
       <c r="C153" s="3" t="n">
-        <v>0</v>
+        <v>0.056</v>
       </c>
       <c r="D153" s="3" t="n">
-        <v>0</v>
+        <v>0.03</v>
       </c>
       <c r="E153" s="3" t="n">
         <v>0</v>
       </c>
       <c r="F153" s="3" t="n">
-        <v>0.058</v>
+        <v>0.038</v>
       </c>
       <c r="G153" s="3" t="n">
         <v>0</v>
@@ -10716,51 +10713,15 @@
         <v>0</v>
       </c>
       <c r="J153" s="4" t="n">
-        <v>0.00348</v>
+        <v>0.00228</v>
       </c>
       <c r="K153" s="3" t="n">
         <f aca="false">SUM(B153:I153)</f>
-        <v>0.058</v>
-      </c>
-    </row>
-    <row r="154" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A154" s="0" t="s">
-        <v>125</v>
-      </c>
-      <c r="B154" s="3" t="n">
-        <v>0.167</v>
-      </c>
-      <c r="C154" s="3" t="n">
-        <v>0.053</v>
-      </c>
-      <c r="D154" s="3" t="n">
-        <v>0.029</v>
-      </c>
-      <c r="E154" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="F154" s="3" t="n">
-        <v>0.038</v>
-      </c>
-      <c r="G154" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="H154" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="I154" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="J154" s="4" t="n">
-        <v>0.00228</v>
-      </c>
-      <c r="K154" s="3" t="n">
-        <f aca="false">SUM(B154:I154)</f>
-        <v>0.287</v>
+        <v>0.3</v>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A3:K154"/>
+  <autoFilter ref="A3:K153"/>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
   <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>

</xml_diff>